<commit_message>
Hacer xgboost con spatial cv
</commit_message>
<xml_diff>
--- a/Seguimiento submissions.xlsx
+++ b/Seguimiento submissions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\luiyi\Dropbox\Lu\Backup\Big data y Machine Learning para Economía Aplicada\Taller-3\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6CF6AD2F-671A-4FA2-9BD7-D8FFD6C16CA9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EE26EE37-B2BF-4BC3-8ACB-71D448065923}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" xr2:uid="{61DA3C93-0847-4C6B-9B33-18547C96FEBD}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="18">
   <si>
     <t xml:space="preserve">Archivo </t>
   </si>
@@ -81,6 +81,36 @@
   </si>
   <si>
     <t xml:space="preserve">Hay una diferencia abislmal entre el error de train y el de generalización. Además, el error de generalización es altísimo, teniendo en cuenta que el promedio de los precios de las propiedades es de 654.534.675. Creo que tiene que ver con la cantidad de observaciones usadas. Se usaron para entrenar, 4.307 observaciones y se evaluó en 10.286. Creo que es mejor tratar primero los NAs y después si reestimar el modelo a ver qué pasa. </t>
+  </si>
+  <si>
+    <t>xgboost11</t>
+  </si>
+  <si>
+    <t>eta = 0.05
+max_depth = 8
+gamma = 0.1
+colsample_bytree = 0.75
+min_child_weight = 20
+subsample = 0.75
+nrounds = 1000</t>
+  </si>
+  <si>
+    <t xml:space="preserve">En esta iteración se buscó en la variable de texto para completar los NAs de área total, construída, baños y cuartos, lo cual disminuyó un tercio los NAs, igual quedan todavía NAs. Además, se crearon variables que contaba los NAs de estas variables para permitirle al xgboost aprender de los missings. Por último, se sacó el logaritmo de los precios. Se puede ver que el error de validación disminuyó, pero el error del train aumentó, lo que podría indicar sobreajuste. También se oberva que, igual que en el caso anterior, la brecha entre el error de validación y de entrenamiento es alta. Lo que puede indicar que las propiedades de chapinero no tienen características silimilares al resto de barrios de Bogotá. </t>
+  </si>
+  <si>
+    <t>xgboost_spatial_cv</t>
+  </si>
+  <si>
+    <t>Todas + lat y lon + estrato</t>
+  </si>
+  <si>
+    <t>eta = 0.05
+max_depth = 8
+gamma = 0.1
+colsample_bytree = 0.75
+min_child_weight = 20
+subsample = 0.75
+nrounds = 500</t>
   </si>
 </sst>
 </file>
@@ -129,7 +159,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
@@ -146,6 +176,12 @@
     </xf>
     <xf numFmtId="4" fontId="1" fillId="2" borderId="0" xfId="1" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -482,12 +518,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A70B91BE-477A-4823-BA77-A1BE7105F8DB}">
-  <dimension ref="A1:G2"/>
+  <dimension ref="A1:G4"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
+    <col min="3" max="3" width="13.81640625" style="8" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="23.36328125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.453125" style="3" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="13.453125" style="3" bestFit="1" customWidth="1"/>
+    <col min="5" max="6" width="13.453125" style="3" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="86.08984375" customWidth="1"/>
   </cols>
   <sheetData>
@@ -498,7 +534,7 @@
       <c r="B1" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="5" t="s">
+      <c r="C1" s="7" t="s">
         <v>2</v>
       </c>
       <c r="D1" s="5" t="s">
@@ -521,7 +557,7 @@
       <c r="B2" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="C2" s="2" t="s">
         <v>9</v>
       </c>
       <c r="D2" s="2" t="s">
@@ -535,6 +571,49 @@
       </c>
       <c r="G2" s="2" t="s">
         <v>11</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" s="1" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
+      <c r="A3" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E3" s="4">
+        <v>112305618</v>
+      </c>
+      <c r="F3" s="4">
+        <v>251808804.86000001</v>
+      </c>
+      <c r="G3" s="2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" s="1" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
+      <c r="A4" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="E4" s="4">
+        <v>135434740</v>
+      </c>
+      <c r="F4" s="4">
+        <v>183644146</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Agregar un xgboost con DTM
</commit_message>
<xml_diff>
--- a/Seguimiento submissions.xlsx
+++ b/Seguimiento submissions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\luiyi\Dropbox\Lu\Backup\Big data y Machine Learning para Economía Aplicada\Taller-3\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F165C59F-8C70-4A0E-A821-CF0ACED40EB2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D45CF8A1-6B74-486F-B822-9AA78E6524E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" xr2:uid="{61DA3C93-0847-4C6B-9B33-18547C96FEBD}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="36">
   <si>
     <t xml:space="preserve">Archivo </t>
   </si>
@@ -173,6 +173,21 @@
 early_stopping = 30
 epochs = 500
 batch_size = 64</t>
+  </si>
+  <si>
+    <t>xgboost_spatial_cv_dtm</t>
+  </si>
+  <si>
+    <t>Todas + lat y lon + estrato + dtm (8978 col)</t>
+  </si>
+  <si>
+    <t>eta = 0.05
+max_depth = 8
+gamma = 0
+colsample_bytree = 0.66
+min_child_weight = 20
+subsample = 0.66
+nrounds = 1000</t>
   </si>
 </sst>
 </file>
@@ -589,10 +604,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A70B91BE-477A-4823-BA77-A1BE7105F8DB}">
-  <dimension ref="A1:G8"/>
+  <dimension ref="A1:G9"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="17.1796875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="20.08984375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="24.90625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="13.81640625" style="8" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="27.08984375" customWidth="1"/>
@@ -715,69 +730,89 @@
         <v>21</v>
       </c>
     </row>
-    <row r="6" spans="1:7" s="9" customFormat="1" ht="116" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:7" s="9" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A6" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="B6" s="9" t="s">
+        <v>8</v>
+      </c>
+      <c r="C6" s="10" t="s">
+        <v>34</v>
+      </c>
+      <c r="D6" s="10" t="s">
+        <v>35</v>
+      </c>
+      <c r="E6" s="11">
+        <v>124554398</v>
+      </c>
+      <c r="F6" s="11">
+        <v>175637962.86000001</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" s="9" customFormat="1" ht="116" x14ac:dyDescent="0.35">
+      <c r="A7" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="B6" s="9" t="s">
+      <c r="B7" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="C6" s="10" t="s">
+      <c r="C7" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="D6" s="10" t="s">
+      <c r="D7" s="10" t="s">
         <v>25</v>
       </c>
-      <c r="E6" s="11">
+      <c r="E7" s="11">
         <v>122142601</v>
       </c>
-      <c r="F6" s="11">
+      <c r="F7" s="11">
         <v>237152443.13</v>
       </c>
-      <c r="G6" s="9" t="s">
+      <c r="G7" s="9" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="7" spans="1:7" s="1" customFormat="1" ht="116" x14ac:dyDescent="0.35">
-      <c r="A7" s="1" t="s">
+    <row r="8" spans="1:7" s="1" customFormat="1" ht="116" x14ac:dyDescent="0.35">
+      <c r="A8" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="B7" s="1" t="s">
+      <c r="B8" s="1" t="s">
         <v>29</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="D7" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="E7" s="4">
-        <v>142369043</v>
-      </c>
-      <c r="F7" s="4">
-        <v>262782527.15000001</v>
-      </c>
-      <c r="G7" s="1" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" s="1" customFormat="1" ht="87" x14ac:dyDescent="0.35">
-      <c r="A8" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="B8" s="1" t="s">
-        <v>31</v>
       </c>
       <c r="C8" s="2" t="s">
         <v>16</v>
       </c>
       <c r="D8" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="E8" s="4">
+        <v>142369043</v>
+      </c>
+      <c r="F8" s="4">
+        <v>262782527.15000001</v>
+      </c>
+      <c r="G8" s="1" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" s="1" customFormat="1" ht="87" x14ac:dyDescent="0.35">
+      <c r="A9" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="D9" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="E8" s="4">
+      <c r="E9" s="4">
         <v>129073151</v>
       </c>
-      <c r="F8" s="4">
+      <c r="F9" s="4">
         <v>238568458.66</v>
       </c>
     </row>

</xml_diff>